<commit_message>
Add anonymized word cloud demo, enrich sample reflections
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/周计划_template.xlsx
+++ b/周计划_template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1963" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1984" uniqueCount="49">
   <si>
     <t>Time</t>
   </si>
@@ -106,25 +106,61 @@
     <t>小目标达成</t>
   </si>
   <si>
+    <t>灵感爆发</t>
+  </si>
+  <si>
+    <t>继续加油</t>
+  </si>
+  <si>
+    <t>心态平稳</t>
+  </si>
+  <si>
+    <t>按部就班</t>
+  </si>
+  <si>
+    <t>需要调整</t>
+  </si>
+  <si>
+    <t>效率很高</t>
+  </si>
+  <si>
+    <t>慢慢来</t>
+  </si>
+  <si>
     <t>有点累</t>
+  </si>
+  <si>
+    <t>日常打卡</t>
+  </si>
+  <si>
+    <t>专注</t>
+  </si>
+  <si>
+    <t>保持节奏</t>
+  </si>
+  <si>
+    <t>还需努力</t>
+  </si>
+  <si>
+    <t>稳步推进</t>
   </si>
   <si>
     <t>收获很大</t>
   </si>
   <si>
+    <t>值得庆祝</t>
+  </si>
+  <si>
+    <t>满血复活</t>
+  </si>
+  <si>
     <t>状态不错</t>
   </si>
   <si>
-    <t>需要调整</t>
+    <t>精力充沛</t>
   </si>
   <si>
-    <t>按部就班</t>
-  </si>
-  <si>
-    <t>专注</t>
-  </si>
-  <si>
-    <t>效率很高</t>
+    <t>小小疲惫</t>
   </si>
 </sst>
 </file>
@@ -699,6 +735,9 @@
       <c r="L5" t="s">
         <v>15</v>
       </c>
+      <c r="M5" t="s">
+        <v>32</v>
+      </c>
       <c r="N5">
         <v>0</v>
       </c>
@@ -741,7 +780,7 @@
         <v>15</v>
       </c>
       <c r="M6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -785,7 +824,7 @@
         <v>15</v>
       </c>
       <c r="M7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -829,7 +868,7 @@
         <v>15</v>
       </c>
       <c r="M8" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N8">
         <v>5</v>
@@ -873,7 +912,7 @@
         <v>15</v>
       </c>
       <c r="M9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -917,7 +956,7 @@
         <v>15</v>
       </c>
       <c r="M10" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N10">
         <v>13</v>
@@ -961,7 +1000,7 @@
         <v>15</v>
       </c>
       <c r="M11" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -1046,7 +1085,7 @@
         <v>15</v>
       </c>
       <c r="M13" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="N13">
         <v>14</v>
@@ -1090,7 +1129,7 @@
         <v>15</v>
       </c>
       <c r="M14" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -1134,7 +1173,7 @@
         <v>27</v>
       </c>
       <c r="M15" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N15">
         <v>0</v>
@@ -1177,6 +1216,9 @@
       <c r="L16" t="s">
         <v>15</v>
       </c>
+      <c r="M16" t="s">
+        <v>32</v>
+      </c>
       <c r="N16">
         <v>0</v>
       </c>
@@ -1219,7 +1261,7 @@
         <v>15</v>
       </c>
       <c r="M17" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -1263,7 +1305,7 @@
         <v>28</v>
       </c>
       <c r="M18" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="N18">
         <v>8</v>
@@ -1307,7 +1349,7 @@
         <v>15</v>
       </c>
       <c r="M19" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="N19">
         <v>0</v>
@@ -1351,7 +1393,7 @@
         <v>15</v>
       </c>
       <c r="M20" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="N20">
         <v>3</v>
@@ -1395,7 +1437,7 @@
         <v>15</v>
       </c>
       <c r="M21" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="N21">
         <v>10</v>
@@ -1439,7 +1481,7 @@
         <v>15</v>
       </c>
       <c r="M22" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N22">
         <v>0</v>
@@ -1483,7 +1525,7 @@
         <v>15</v>
       </c>
       <c r="M23" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N23">
         <v>8</v>
@@ -1526,6 +1568,9 @@
       <c r="L24" t="s">
         <v>15</v>
       </c>
+      <c r="M24" t="s">
+        <v>32</v>
+      </c>
       <c r="N24">
         <v>0</v>
       </c>
@@ -1568,7 +1613,7 @@
         <v>15</v>
       </c>
       <c r="M25" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="N25">
         <v>12</v>
@@ -1612,7 +1657,7 @@
         <v>15</v>
       </c>
       <c r="M26" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N26">
         <v>0</v>
@@ -1656,7 +1701,7 @@
         <v>15</v>
       </c>
       <c r="M27" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="N27">
         <v>0</v>
@@ -1700,7 +1745,7 @@
         <v>15</v>
       </c>
       <c r="M28" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="N28">
         <v>0</v>
@@ -1744,7 +1789,7 @@
         <v>15</v>
       </c>
       <c r="M29" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="N29">
         <v>28</v>
@@ -1788,7 +1833,7 @@
         <v>15</v>
       </c>
       <c r="M30" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N30">
         <v>0</v>
@@ -1832,7 +1877,7 @@
         <v>15</v>
       </c>
       <c r="M31" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N31">
         <v>0</v>
@@ -1876,7 +1921,7 @@
         <v>27</v>
       </c>
       <c r="M32" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="N32">
         <v>0</v>
@@ -1961,7 +2006,7 @@
         <v>15</v>
       </c>
       <c r="M34" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="N34">
         <v>0</v>
@@ -2005,7 +2050,7 @@
         <v>15</v>
       </c>
       <c r="M35" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N35">
         <v>0</v>
@@ -2049,7 +2094,7 @@
         <v>15</v>
       </c>
       <c r="M36" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="N36">
         <v>0</v>
@@ -2093,7 +2138,7 @@
         <v>15</v>
       </c>
       <c r="M37" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N37">
         <v>0</v>
@@ -2137,7 +2182,7 @@
         <v>15</v>
       </c>
       <c r="M38" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="N38">
         <v>0</v>
@@ -2181,7 +2226,7 @@
         <v>15</v>
       </c>
       <c r="M39" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="N39">
         <v>17</v>
@@ -2225,7 +2270,7 @@
         <v>15</v>
       </c>
       <c r="M40" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N40">
         <v>28</v>
@@ -2269,7 +2314,7 @@
         <v>15</v>
       </c>
       <c r="M41" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N41">
         <v>0</v>
@@ -2313,7 +2358,7 @@
         <v>15</v>
       </c>
       <c r="M42" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="N42">
         <v>0</v>
@@ -2357,7 +2402,7 @@
         <v>15</v>
       </c>
       <c r="M43" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="N43">
         <v>3</v>
@@ -2445,7 +2490,7 @@
         <v>15</v>
       </c>
       <c r="M45" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N45">
         <v>0</v>
@@ -2489,7 +2534,7 @@
         <v>15</v>
       </c>
       <c r="M46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N46">
         <v>25</v>
@@ -2533,7 +2578,7 @@
         <v>15</v>
       </c>
       <c r="M47" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="N47">
         <v>14</v>
@@ -2577,7 +2622,7 @@
         <v>28</v>
       </c>
       <c r="M48" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="N48">
         <v>0</v>
@@ -2621,7 +2666,7 @@
         <v>15</v>
       </c>
       <c r="M49" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N49">
         <v>0</v>
@@ -2665,7 +2710,7 @@
         <v>15</v>
       </c>
       <c r="M50" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N50">
         <v>0</v>
@@ -2709,7 +2754,7 @@
         <v>15</v>
       </c>
       <c r="M51" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N51">
         <v>0</v>
@@ -2753,7 +2798,7 @@
         <v>15</v>
       </c>
       <c r="M52" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="N52">
         <v>0</v>
@@ -2797,7 +2842,7 @@
         <v>15</v>
       </c>
       <c r="M53" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="N53">
         <v>1</v>
@@ -2841,7 +2886,7 @@
         <v>15</v>
       </c>
       <c r="M54" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N54">
         <v>0</v>
@@ -2885,7 +2930,7 @@
         <v>15</v>
       </c>
       <c r="M55" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="N55">
         <v>25</v>
@@ -2929,7 +2974,7 @@
         <v>15</v>
       </c>
       <c r="M56" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N56">
         <v>0</v>
@@ -2973,7 +3018,7 @@
         <v>15</v>
       </c>
       <c r="M57" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N57">
         <v>16</v>
@@ -3017,7 +3062,7 @@
         <v>15</v>
       </c>
       <c r="M58" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="N58">
         <v>0</v>
@@ -3061,7 +3106,7 @@
         <v>15</v>
       </c>
       <c r="M59" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N59">
         <v>0</v>
@@ -3105,7 +3150,7 @@
         <v>15</v>
       </c>
       <c r="M60" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N60">
         <v>0</v>
@@ -3149,7 +3194,7 @@
         <v>15</v>
       </c>
       <c r="M61" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N61">
         <v>0</v>
@@ -3193,7 +3238,7 @@
         <v>15</v>
       </c>
       <c r="M62" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N62">
         <v>0</v>
@@ -3236,6 +3281,9 @@
       <c r="L63" t="s">
         <v>15</v>
       </c>
+      <c r="M63" t="s">
+        <v>47</v>
+      </c>
       <c r="N63">
         <v>0</v>
       </c>
@@ -3278,7 +3326,7 @@
         <v>15</v>
       </c>
       <c r="M64" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N64">
         <v>0</v>
@@ -3322,7 +3370,7 @@
         <v>15</v>
       </c>
       <c r="M65" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N65">
         <v>0</v>
@@ -3366,7 +3414,7 @@
         <v>15</v>
       </c>
       <c r="M66" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N66">
         <v>15</v>
@@ -3410,7 +3458,7 @@
         <v>15</v>
       </c>
       <c r="M67" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N67">
         <v>0</v>
@@ -3454,7 +3502,7 @@
         <v>15</v>
       </c>
       <c r="M68" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N68">
         <v>0</v>
@@ -3498,7 +3546,7 @@
         <v>15</v>
       </c>
       <c r="M69" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N69">
         <v>17</v>
@@ -3542,7 +3590,7 @@
         <v>15</v>
       </c>
       <c r="M70" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="N70">
         <v>0</v>
@@ -3586,7 +3634,7 @@
         <v>15</v>
       </c>
       <c r="M71" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N71">
         <v>27</v>
@@ -3629,6 +3677,9 @@
       <c r="L72" t="s">
         <v>15</v>
       </c>
+      <c r="M72" t="s">
+        <v>47</v>
+      </c>
       <c r="N72">
         <v>17</v>
       </c>
@@ -3670,6 +3721,9 @@
       <c r="L73" t="s">
         <v>28</v>
       </c>
+      <c r="M73" t="s">
+        <v>32</v>
+      </c>
       <c r="N73">
         <v>0</v>
       </c>
@@ -3712,7 +3766,7 @@
         <v>15</v>
       </c>
       <c r="M74" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="N74">
         <v>9</v>
@@ -3756,7 +3810,7 @@
         <v>15</v>
       </c>
       <c r="M75" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N75">
         <v>14</v>
@@ -3799,6 +3853,9 @@
       <c r="L76" t="s">
         <v>15</v>
       </c>
+      <c r="M76" t="s">
+        <v>47</v>
+      </c>
       <c r="N76">
         <v>0</v>
       </c>
@@ -3841,7 +3898,7 @@
         <v>15</v>
       </c>
       <c r="M77" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N77">
         <v>13</v>
@@ -3885,7 +3942,7 @@
         <v>15</v>
       </c>
       <c r="M78" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="N78">
         <v>0</v>
@@ -3929,7 +3986,7 @@
         <v>15</v>
       </c>
       <c r="M79" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="N79">
         <v>0</v>
@@ -3973,7 +4030,7 @@
         <v>15</v>
       </c>
       <c r="M80" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="N80">
         <v>13</v>
@@ -4016,6 +4073,9 @@
       <c r="L81" t="s">
         <v>15</v>
       </c>
+      <c r="M81" t="s">
+        <v>47</v>
+      </c>
       <c r="N81">
         <v>0</v>
       </c>
@@ -4057,6 +4117,9 @@
       <c r="L82" t="s">
         <v>15</v>
       </c>
+      <c r="M82" t="s">
+        <v>47</v>
+      </c>
       <c r="N82">
         <v>0</v>
       </c>
@@ -4099,7 +4162,7 @@
         <v>15</v>
       </c>
       <c r="M83" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="N83">
         <v>0</v>
@@ -4187,7 +4250,7 @@
         <v>15</v>
       </c>
       <c r="M85" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="N85">
         <v>0</v>
@@ -4230,6 +4293,9 @@
       <c r="L86" t="s">
         <v>15</v>
       </c>
+      <c r="M86" t="s">
+        <v>47</v>
+      </c>
       <c r="N86">
         <v>0</v>
       </c>
@@ -4272,7 +4338,7 @@
         <v>15</v>
       </c>
       <c r="M87" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N87">
         <v>4</v>
@@ -4357,7 +4423,7 @@
         <v>15</v>
       </c>
       <c r="M89" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="N89">
         <v>0</v>
@@ -4486,7 +4552,7 @@
         <v>15</v>
       </c>
       <c r="M92" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N92">
         <v>0</v>
@@ -4530,7 +4596,7 @@
         <v>15</v>
       </c>
       <c r="M93" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N93">
         <v>0</v>
@@ -4574,7 +4640,7 @@
         <v>15</v>
       </c>
       <c r="M94" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="N94">
         <v>0</v>
@@ -4618,7 +4684,7 @@
         <v>29</v>
       </c>
       <c r="M95" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="N95">
         <v>0</v>
@@ -4662,7 +4728,7 @@
         <v>15</v>
       </c>
       <c r="M96" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N96">
         <v>16</v>
@@ -4706,7 +4772,7 @@
         <v>15</v>
       </c>
       <c r="M97" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="N97">
         <v>0</v>
@@ -4750,7 +4816,7 @@
         <v>15</v>
       </c>
       <c r="M98" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N98">
         <v>19</v>
@@ -4793,6 +4859,9 @@
       <c r="L99" t="s">
         <v>15</v>
       </c>
+      <c r="M99" t="s">
+        <v>47</v>
+      </c>
       <c r="N99">
         <v>0</v>
       </c>
@@ -4879,7 +4948,7 @@
         <v>15</v>
       </c>
       <c r="M101" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="N101">
         <v>0</v>
@@ -4967,7 +5036,7 @@
         <v>15</v>
       </c>
       <c r="M103" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="N103">
         <v>0</v>
@@ -5011,7 +5080,7 @@
         <v>15</v>
       </c>
       <c r="M104" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N104">
         <v>13</v>
@@ -5055,7 +5124,7 @@
         <v>15</v>
       </c>
       <c r="M105" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N105">
         <v>0</v>
@@ -5099,7 +5168,7 @@
         <v>15</v>
       </c>
       <c r="M106" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N106">
         <v>5</v>
@@ -5187,7 +5256,7 @@
         <v>15</v>
       </c>
       <c r="M108" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N108">
         <v>0</v>
@@ -5231,7 +5300,7 @@
         <v>15</v>
       </c>
       <c r="M109" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="N109">
         <v>18</v>
@@ -5274,6 +5343,9 @@
       <c r="L110" t="s">
         <v>15</v>
       </c>
+      <c r="M110" t="s">
+        <v>32</v>
+      </c>
       <c r="N110">
         <v>0</v>
       </c>
@@ -5315,6 +5387,9 @@
       <c r="L111" t="s">
         <v>15</v>
       </c>
+      <c r="M111" t="s">
+        <v>47</v>
+      </c>
       <c r="N111">
         <v>0</v>
       </c>
@@ -5356,6 +5431,9 @@
       <c r="L112" t="s">
         <v>15</v>
       </c>
+      <c r="M112" t="s">
+        <v>32</v>
+      </c>
       <c r="N112">
         <v>0</v>
       </c>
@@ -5398,7 +5476,7 @@
         <v>15</v>
       </c>
       <c r="M113" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="N113">
         <v>18</v>
@@ -5483,7 +5561,7 @@
         <v>15</v>
       </c>
       <c r="M115" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="N115">
         <v>0</v>
@@ -5527,7 +5605,7 @@
         <v>15</v>
       </c>
       <c r="M116" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="N116">
         <v>0</v>
@@ -5571,7 +5649,7 @@
         <v>15</v>
       </c>
       <c r="M117" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="N117">
         <v>0</v>
@@ -5615,7 +5693,7 @@
         <v>27</v>
       </c>
       <c r="M118" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="N118">
         <v>0</v>
@@ -5659,7 +5737,7 @@
         <v>15</v>
       </c>
       <c r="M119" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N119">
         <v>29</v>
@@ -5703,7 +5781,7 @@
         <v>15</v>
       </c>
       <c r="M120" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="N120">
         <v>0</v>
@@ -5747,7 +5825,7 @@
         <v>15</v>
       </c>
       <c r="M121" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N121">
         <v>0</v>
@@ -5791,7 +5869,7 @@
         <v>15</v>
       </c>
       <c r="M122" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N122">
         <v>17</v>
@@ -5835,7 +5913,7 @@
         <v>15</v>
       </c>
       <c r="M123" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="N123">
         <v>19</v>
@@ -5879,7 +5957,7 @@
         <v>15</v>
       </c>
       <c r="M124" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="N124">
         <v>0</v>
@@ -5923,7 +6001,7 @@
         <v>15</v>
       </c>
       <c r="M125" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N125">
         <v>0</v>
@@ -5967,7 +6045,7 @@
         <v>15</v>
       </c>
       <c r="M126" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N126">
         <v>0</v>
@@ -6011,7 +6089,7 @@
         <v>15</v>
       </c>
       <c r="M127" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="N127">
         <v>0</v>
@@ -6098,6 +6176,9 @@
       <c r="L129" t="s">
         <v>15</v>
       </c>
+      <c r="M129" t="s">
+        <v>47</v>
+      </c>
       <c r="N129">
         <v>0</v>
       </c>
@@ -6183,6 +6264,9 @@
       <c r="L131" t="s">
         <v>15</v>
       </c>
+      <c r="M131" t="s">
+        <v>32</v>
+      </c>
       <c r="N131">
         <v>0</v>
       </c>
@@ -6224,6 +6308,9 @@
       <c r="L132" t="s">
         <v>15</v>
       </c>
+      <c r="M132" t="s">
+        <v>47</v>
+      </c>
       <c r="N132">
         <v>0</v>
       </c>
@@ -6266,7 +6353,7 @@
         <v>15</v>
       </c>
       <c r="M133" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N133">
         <v>10</v>
@@ -6310,7 +6397,7 @@
         <v>27</v>
       </c>
       <c r="M134" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="N134">
         <v>0</v>
@@ -6354,7 +6441,7 @@
         <v>15</v>
       </c>
       <c r="M135" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="N135">
         <v>0</v>
@@ -6439,7 +6526,7 @@
         <v>15</v>
       </c>
       <c r="M137" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N137">
         <v>0</v>
@@ -6483,7 +6570,7 @@
         <v>15</v>
       </c>
       <c r="M138" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N138">
         <v>0</v>
@@ -6568,7 +6655,7 @@
         <v>15</v>
       </c>
       <c r="M140" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="N140">
         <v>0</v>
@@ -6612,7 +6699,7 @@
         <v>15</v>
       </c>
       <c r="M141" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N141">
         <v>0</v>
@@ -6744,7 +6831,7 @@
         <v>15</v>
       </c>
       <c r="M144" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N144">
         <v>0</v>
@@ -6788,7 +6875,7 @@
         <v>15</v>
       </c>
       <c r="M145" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N145">
         <v>0</v>
@@ -6832,7 +6919,7 @@
         <v>15</v>
       </c>
       <c r="M146" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="N146">
         <v>5</v>
@@ -6875,6 +6962,9 @@
       <c r="L147" t="s">
         <v>15</v>
       </c>
+      <c r="M147" t="s">
+        <v>32</v>
+      </c>
       <c r="N147">
         <v>0</v>
       </c>
@@ -6917,7 +7007,7 @@
         <v>15</v>
       </c>
       <c r="M148" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="N148">
         <v>0</v>
@@ -6961,7 +7051,7 @@
         <v>15</v>
       </c>
       <c r="M149" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N149">
         <v>0</v>
@@ -7005,7 +7095,7 @@
         <v>15</v>
       </c>
       <c r="M150" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N150">
         <v>9</v>
@@ -7090,7 +7180,7 @@
         <v>15</v>
       </c>
       <c r="M152" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="N152">
         <v>6</v>
@@ -7134,7 +7224,7 @@
         <v>15</v>
       </c>
       <c r="M153" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N153">
         <v>0</v>
@@ -7178,7 +7268,7 @@
         <v>15</v>
       </c>
       <c r="M154" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N154">
         <v>19</v>
@@ -7221,6 +7311,9 @@
       <c r="L155" t="s">
         <v>15</v>
       </c>
+      <c r="M155" t="s">
+        <v>47</v>
+      </c>
       <c r="N155">
         <v>0</v>
       </c>
@@ -7263,7 +7356,7 @@
         <v>15</v>
       </c>
       <c r="M156" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="N156">
         <v>0</v>
@@ -7307,7 +7400,7 @@
         <v>15</v>
       </c>
       <c r="M157" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N157">
         <v>0</v>
@@ -7351,7 +7444,7 @@
         <v>15</v>
       </c>
       <c r="M158" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N158">
         <v>0</v>
@@ -7436,7 +7529,7 @@
         <v>28</v>
       </c>
       <c r="M160" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N160">
         <v>0</v>
@@ -7480,7 +7573,7 @@
         <v>15</v>
       </c>
       <c r="M161" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N161">
         <v>0</v>
@@ -7524,7 +7617,7 @@
         <v>15</v>
       </c>
       <c r="M162" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N162">
         <v>0</v>
@@ -7568,7 +7661,7 @@
         <v>27</v>
       </c>
       <c r="M163" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N163">
         <v>0</v>
@@ -7612,7 +7705,7 @@
         <v>15</v>
       </c>
       <c r="M164" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N164">
         <v>0</v>
@@ -7656,7 +7749,7 @@
         <v>15</v>
       </c>
       <c r="M165" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="N165">
         <v>0</v>
@@ -7700,7 +7793,7 @@
         <v>15</v>
       </c>
       <c r="M166" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N166">
         <v>19</v>
@@ -7744,7 +7837,7 @@
         <v>15</v>
       </c>
       <c r="M167" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="N167">
         <v>12</v>
@@ -7788,7 +7881,7 @@
         <v>15</v>
       </c>
       <c r="M168" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="N168">
         <v>0</v>
@@ -7831,6 +7924,9 @@
       <c r="L169" t="s">
         <v>15</v>
       </c>
+      <c r="M169" t="s">
+        <v>47</v>
+      </c>
       <c r="N169">
         <v>0</v>
       </c>
@@ -7873,7 +7969,7 @@
         <v>15</v>
       </c>
       <c r="M170" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N170">
         <v>0</v>
@@ -7917,7 +8013,7 @@
         <v>15</v>
       </c>
       <c r="M171" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="N171">
         <v>0</v>
@@ -7960,6 +8056,9 @@
       <c r="L172" t="s">
         <v>15</v>
       </c>
+      <c r="M172" t="s">
+        <v>47</v>
+      </c>
       <c r="N172">
         <v>29</v>
       </c>
@@ -8002,7 +8101,7 @@
         <v>15</v>
       </c>
       <c r="M173" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="N173">
         <v>0</v>
@@ -8046,7 +8145,7 @@
         <v>15</v>
       </c>
       <c r="M174" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="N174">
         <v>8</v>
@@ -8090,7 +8189,7 @@
         <v>15</v>
       </c>
       <c r="M175" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="N175">
         <v>18</v>
@@ -8134,7 +8233,7 @@
         <v>15</v>
       </c>
       <c r="M176" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N176">
         <v>0</v>
@@ -8178,7 +8277,7 @@
         <v>15</v>
       </c>
       <c r="M177" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="N177">
         <v>0</v>
@@ -8222,7 +8321,7 @@
         <v>15</v>
       </c>
       <c r="M178" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="N178">
         <v>0</v>
@@ -8266,7 +8365,7 @@
         <v>15</v>
       </c>
       <c r="M179" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N179">
         <v>0</v>
@@ -8310,7 +8409,7 @@
         <v>15</v>
       </c>
       <c r="M180" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N180">
         <v>0</v>
@@ -8354,7 +8453,7 @@
         <v>15</v>
       </c>
       <c r="M181" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N181">
         <v>0</v>

</xml_diff>